<commit_message>
Update RP2350 PCB(A) files
</commit_message>
<xml_diff>
--- a/pcb/rp2350/mainboard/pcb assembly JLC/p2_pcb_rp2350_v1_4_bom_JLC.xlsx
+++ b/pcb/rp2350/mainboard/pcb assembly JLC/p2_pcb_rp2350_v1_4_bom_JLC.xlsx
@@ -14,12 +14,12 @@
   <sheets>
     <sheet name="p2_pcb_rp2350_v1_4_bom_JLC" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="0" iterateDelta="1E-4"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="158">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="160">
   <si>
     <t>Comment</t>
   </si>
@@ -288,9 +288,6 @@
     <t>U12</t>
   </si>
   <si>
-    <t>C5333729</t>
-  </si>
-  <si>
     <t>Y1</t>
   </si>
   <si>
@@ -321,9 +318,6 @@
     <t>J7</t>
   </si>
   <si>
-    <t>C262230</t>
-  </si>
-  <si>
     <t>SW9</t>
   </si>
   <si>
@@ -333,9 +327,6 @@
     <t>SW10, SW11</t>
   </si>
   <si>
-    <t>C2886894</t>
-  </si>
-  <si>
     <t>JLCPCB Part #</t>
   </si>
   <si>
@@ -369,9 +360,6 @@
     <t>PJ-242</t>
   </si>
   <si>
-    <t>AFC07-S05ECC-00</t>
-  </si>
-  <si>
     <t>TL3330AF260QG</t>
   </si>
   <si>
@@ -384,9 +372,6 @@
     <t>C17593</t>
   </si>
   <si>
-    <t>C17594</t>
-  </si>
-  <si>
     <t>C25611</t>
   </si>
   <si>
@@ -396,9 +381,6 @@
     <t>C17630</t>
   </si>
   <si>
-    <t>C17513</t>
-  </si>
-  <si>
     <t>C17393</t>
   </si>
   <si>
@@ -432,9 +414,6 @@
     <t>C53884</t>
   </si>
   <si>
-    <t>APS6404L-3SQR-SN</t>
-  </si>
-  <si>
     <t>W25Q128JVSQ</t>
   </si>
   <si>
@@ -456,9 +435,6 @@
     <t>F-FPC0M40P-C310</t>
   </si>
   <si>
-    <t>C2886897</t>
-  </si>
-  <si>
     <t>20k 1%</t>
   </si>
   <si>
@@ -493,6 +469,36 @@
   </si>
   <si>
     <t>Alternative</t>
+  </si>
+  <si>
+    <t>C92584</t>
+  </si>
+  <si>
+    <t>C5333729 (3SQR)</t>
+  </si>
+  <si>
+    <t>C3028887</t>
+  </si>
+  <si>
+    <t>APS6404L-3SQN-SN</t>
+  </si>
+  <si>
+    <t>C262578</t>
+  </si>
+  <si>
+    <t>AFC07-S05ECA-00</t>
+  </si>
+  <si>
+    <t>C5261054</t>
+  </si>
+  <si>
+    <t>C25100</t>
+  </si>
+  <si>
+    <t>C11702</t>
+  </si>
+  <si>
+    <t>C410364</t>
   </si>
 </sst>
 </file>
@@ -1323,10 +1329,10 @@
         <v>2</v>
       </c>
       <c r="D1" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="E1" t="s">
-        <v>157</v>
+        <v>149</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.55000000000000004">
@@ -1368,7 +1374,7 @@
         <v>12</v>
       </c>
       <c r="D4" t="s">
-        <v>121</v>
+        <v>157</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.55000000000000004">
@@ -1382,7 +1388,7 @@
         <v>5</v>
       </c>
       <c r="D5" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.55000000000000004">
@@ -1396,7 +1402,7 @@
         <v>5</v>
       </c>
       <c r="D6" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.55000000000000004">
@@ -1438,7 +1444,7 @@
         <v>5</v>
       </c>
       <c r="D9" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.55000000000000004">
@@ -1452,7 +1458,7 @@
         <v>12</v>
       </c>
       <c r="D10" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.55000000000000004">
@@ -1466,12 +1472,12 @@
         <v>12</v>
       </c>
       <c r="D11" t="s">
-        <v>125</v>
+        <v>158</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A12" t="s">
-        <v>139</v>
+        <v>132</v>
       </c>
       <c r="B12" t="s">
         <v>27</v>
@@ -1480,7 +1486,7 @@
         <v>5</v>
       </c>
       <c r="D12" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.55000000000000004">
@@ -1494,7 +1500,7 @@
         <v>5</v>
       </c>
       <c r="D13" t="s">
-        <v>136</v>
+        <v>130</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.55000000000000004">
@@ -1508,21 +1514,21 @@
         <v>5</v>
       </c>
       <c r="D14" t="s">
-        <v>126</v>
+        <v>120</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A15" t="s">
-        <v>146</v>
+        <v>138</v>
       </c>
       <c r="B15" t="s">
-        <v>147</v>
+        <v>139</v>
       </c>
       <c r="C15" t="s">
         <v>5</v>
       </c>
       <c r="D15" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.55000000000000004">
@@ -1536,7 +1542,7 @@
         <v>5</v>
       </c>
       <c r="D16" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.55000000000000004">
@@ -1544,13 +1550,13 @@
         <v>34</v>
       </c>
       <c r="B17" t="s">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="C17" t="s">
         <v>5</v>
       </c>
       <c r="D17" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.55000000000000004">
@@ -1592,7 +1598,7 @@
         <v>5</v>
       </c>
       <c r="D20" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.55000000000000004">
@@ -1606,7 +1612,7 @@
         <v>5</v>
       </c>
       <c r="D21" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.55000000000000004">
@@ -1620,7 +1626,7 @@
         <v>5</v>
       </c>
       <c r="D22" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.55000000000000004">
@@ -1648,7 +1654,7 @@
         <v>12</v>
       </c>
       <c r="D24" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.55000000000000004">
@@ -1662,7 +1668,7 @@
         <v>12</v>
       </c>
       <c r="D25" t="s">
-        <v>134</v>
+        <v>128</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.55000000000000004">
@@ -1676,12 +1682,12 @@
         <v>5</v>
       </c>
       <c r="D26" t="s">
-        <v>135</v>
+        <v>129</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A27" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="B27" t="s">
         <v>54</v>
@@ -1695,7 +1701,7 @@
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A28" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="B28" t="s">
         <v>57</v>
@@ -1709,7 +1715,7 @@
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A29" s="1" t="s">
-        <v>153</v>
+        <v>145</v>
       </c>
       <c r="B29" t="s">
         <v>59</v>
@@ -1720,7 +1726,7 @@
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A30" t="s">
-        <v>152</v>
+        <v>144</v>
       </c>
       <c r="B30" t="s">
         <v>61</v>
@@ -1734,7 +1740,7 @@
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A31" t="s">
-        <v>155</v>
+        <v>147</v>
       </c>
       <c r="B31" t="s">
         <v>63</v>
@@ -1743,15 +1749,15 @@
         <v>5020</v>
       </c>
       <c r="D31" t="s">
-        <v>154</v>
+        <v>146</v>
       </c>
       <c r="E31" t="s">
-        <v>156</v>
+        <v>148</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A32" t="s">
-        <v>140</v>
+        <v>133</v>
       </c>
       <c r="B32" t="s">
         <v>64</v>
@@ -1760,10 +1766,13 @@
         <v>65</v>
       </c>
       <c r="D32" t="s">
+        <v>156</v>
+      </c>
+      <c r="E32" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A33" t="s">
         <v>67</v>
       </c>
@@ -1777,7 +1786,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A34" t="s">
         <v>71</v>
       </c>
@@ -1791,7 +1800,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A35" t="s">
         <v>74</v>
       </c>
@@ -1805,9 +1814,9 @@
         <v>76</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A36" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="B36" t="s">
         <v>77</v>
@@ -1816,9 +1825,9 @@
         <v>78</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A37" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="B37" t="s">
         <v>79</v>
@@ -1827,9 +1836,9 @@
         <v>80</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A38" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="B38" t="s">
         <v>81</v>
@@ -1838,20 +1847,20 @@
         <v>82</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A39" t="s">
-        <v>141</v>
+        <v>134</v>
       </c>
       <c r="B39" t="s">
         <v>83</v>
       </c>
       <c r="D39" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A40" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="B40" t="s">
         <v>84</v>
@@ -1860,9 +1869,9 @@
         <v>85</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A41" t="s">
-        <v>138</v>
+        <v>131</v>
       </c>
       <c r="B41" t="s">
         <v>86</v>
@@ -1871,117 +1880,120 @@
         <v>87</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A42" t="s">
-        <v>137</v>
+        <v>153</v>
       </c>
       <c r="B42" t="s">
         <v>88</v>
       </c>
       <c r="D42" t="s">
+        <v>152</v>
+      </c>
+      <c r="E42" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A43" t="s">
+        <v>109</v>
+      </c>
+      <c r="B43" t="s">
         <v>89</v>
       </c>
-    </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.55000000000000004">
-      <c r="A43" t="s">
+      <c r="D43" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A44" t="s">
+        <v>137</v>
+      </c>
+      <c r="B44" t="s">
+        <v>91</v>
+      </c>
+      <c r="D44" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A45" t="s">
+        <v>110</v>
+      </c>
+      <c r="B45" t="s">
+        <v>92</v>
+      </c>
+      <c r="D45" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A46" t="s">
+        <v>111</v>
+      </c>
+      <c r="B46" t="s">
+        <v>94</v>
+      </c>
+      <c r="D46" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A47" t="s">
         <v>112</v>
       </c>
-      <c r="B43" t="s">
-        <v>90</v>
-      </c>
-      <c r="D43" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.55000000000000004">
-      <c r="A44" t="s">
-        <v>144</v>
-      </c>
-      <c r="B44" t="s">
-        <v>92</v>
-      </c>
-      <c r="D44" t="s">
+      <c r="B47" t="s">
+        <v>96</v>
+      </c>
+      <c r="D47" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A48" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.55000000000000004">
-      <c r="A45" t="s">
-        <v>113</v>
-      </c>
-      <c r="B45" t="s">
-        <v>93</v>
-      </c>
-      <c r="D45" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.55000000000000004">
-      <c r="A46" t="s">
-        <v>114</v>
-      </c>
-      <c r="B46" t="s">
-        <v>95</v>
-      </c>
-      <c r="D46" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.55000000000000004">
-      <c r="A47" t="s">
-        <v>115</v>
-      </c>
-      <c r="B47" t="s">
-        <v>97</v>
-      </c>
-      <c r="D47" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.55000000000000004">
-      <c r="A48" t="s">
-        <v>151</v>
-      </c>
       <c r="B48" t="s">
-        <v>149</v>
+        <v>141</v>
       </c>
       <c r="D48" t="s">
-        <v>150</v>
+        <v>142</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A49" t="s">
-        <v>116</v>
+        <v>155</v>
       </c>
       <c r="B49" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D49" t="s">
-        <v>100</v>
+        <v>154</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A50" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="B50" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="D50" t="s">
-        <v>102</v>
+        <v>159</v>
+      </c>
+      <c r="E50" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A51" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="B51" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="D51" t="s">
-        <v>104</v>
-      </c>
-      <c r="E51" t="s">
-        <v>145</v>
+        <v>150</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update 3D printed files
</commit_message>
<xml_diff>
--- a/pcb/rp2350/mainboard/pcb assembly JLC/p2_pcb_rp2350_v1_4_bom_JLC.xlsx
+++ b/pcb/rp2350/mainboard/pcb assembly JLC/p2_pcb_rp2350_v1_4_bom_JLC.xlsx
@@ -423,12 +423,6 @@
     <t>DMG2305UX-7</t>
   </si>
   <si>
-    <t>TP4057</t>
-  </si>
-  <si>
-    <t>C12044</t>
-  </si>
-  <si>
     <t>C132511</t>
   </si>
   <si>
@@ -499,6 +493,12 @@
   </si>
   <si>
     <t>C410364</t>
+  </si>
+  <si>
+    <t>TP4054</t>
+  </si>
+  <si>
+    <t>C32574</t>
   </si>
 </sst>
 </file>
@@ -1332,7 +1332,7 @@
         <v>102</v>
       </c>
       <c r="E1" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.55000000000000004">
@@ -1374,7 +1374,7 @@
         <v>12</v>
       </c>
       <c r="D4" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.55000000000000004">
@@ -1472,7 +1472,7 @@
         <v>12</v>
       </c>
       <c r="D11" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.55000000000000004">
@@ -1519,10 +1519,10 @@
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A15" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="B15" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="C15" t="s">
         <v>5</v>
@@ -1550,7 +1550,7 @@
         <v>34</v>
       </c>
       <c r="B17" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="C17" t="s">
         <v>5</v>
@@ -1715,7 +1715,7 @@
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A29" s="1" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="B29" t="s">
         <v>59</v>
@@ -1726,7 +1726,7 @@
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A30" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="B30" t="s">
         <v>61</v>
@@ -1740,7 +1740,7 @@
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A31" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="B31" t="s">
         <v>63</v>
@@ -1749,10 +1749,10 @@
         <v>5020</v>
       </c>
       <c r="D31" t="s">
+        <v>144</v>
+      </c>
+      <c r="E31" t="s">
         <v>146</v>
-      </c>
-      <c r="E31" t="s">
-        <v>148</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.55000000000000004">
@@ -1766,7 +1766,7 @@
         <v>65</v>
       </c>
       <c r="D32" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="E32" t="s">
         <v>66</v>
@@ -1849,13 +1849,13 @@
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A39" t="s">
-        <v>134</v>
+        <v>158</v>
       </c>
       <c r="B39" t="s">
         <v>83</v>
       </c>
       <c r="D39" t="s">
-        <v>135</v>
+        <v>159</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.55000000000000004">
@@ -1882,16 +1882,16 @@
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A42" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="B42" t="s">
         <v>88</v>
       </c>
       <c r="D42" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="E42" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.55000000000000004">
@@ -1907,13 +1907,13 @@
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A44" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="B44" t="s">
         <v>91</v>
       </c>
       <c r="D44" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.55000000000000004">
@@ -1951,24 +1951,24 @@
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A48" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="B48" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="D48" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A49" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="B49" t="s">
         <v>98</v>
       </c>
       <c r="D49" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.55000000000000004">
@@ -1979,7 +1979,7 @@
         <v>99</v>
       </c>
       <c r="D50" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="E50" t="s">
         <v>100</v>
@@ -1993,7 +1993,7 @@
         <v>101</v>
       </c>
       <c r="D51" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix wrong capacitor value in JLCPCB BOM
</commit_message>
<xml_diff>
--- a/pcb/rp2350/mainboard/pcb assembly JLC/p2_pcb_rp2350_v1_4_bom_JLC.xlsx
+++ b/pcb/rp2350/mainboard/pcb assembly JLC/p2_pcb_rp2350_v1_4_bom_JLC.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8394"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8400"/>
   </bookViews>
   <sheets>
     <sheet name="p2_pcb_rp2350_v1_4_bom_JLC" sheetId="1" r:id="rId1"/>
@@ -138,9 +138,6 @@
     <t>C9, C14, C16, C17</t>
   </si>
   <si>
-    <t>C1548</t>
-  </si>
-  <si>
     <t>10 uF</t>
   </si>
   <si>
@@ -499,6 +496,9 @@
   </si>
   <si>
     <t>C32574</t>
+  </si>
+  <si>
+    <t>C23733</t>
   </si>
 </sst>
 </file>
@@ -1312,13 +1312,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:E51"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="43.89453125" customWidth="1"/>
-    <col min="3" max="3" width="35.83984375" customWidth="1"/>
+    <col min="1" max="1" width="43.85546875" customWidth="1"/>
+    <col min="2" max="2" width="53.42578125" customWidth="1"/>
+    <col min="3" max="3" width="35.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1329,13 +1330,13 @@
         <v>2</v>
       </c>
       <c r="D1" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E1" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -1349,7 +1350,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>7</v>
       </c>
@@ -1363,7 +1364,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>10</v>
       </c>
@@ -1374,10 +1375,10 @@
         <v>12</v>
       </c>
       <c r="D4" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>13</v>
       </c>
@@ -1388,10 +1389,10 @@
         <v>5</v>
       </c>
       <c r="D5" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>15</v>
       </c>
@@ -1402,10 +1403,10 @@
         <v>5</v>
       </c>
       <c r="D6" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>17</v>
       </c>
@@ -1419,7 +1420,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>17</v>
       </c>
@@ -1433,7 +1434,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>21</v>
       </c>
@@ -1444,10 +1445,10 @@
         <v>5</v>
       </c>
       <c r="D9" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>23</v>
       </c>
@@ -1458,10 +1459,10 @@
         <v>12</v>
       </c>
       <c r="D10" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>25</v>
       </c>
@@ -1472,12 +1473,12 @@
         <v>12</v>
       </c>
       <c r="D11" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B12" t="s">
         <v>27</v>
@@ -1486,10 +1487,10 @@
         <v>5</v>
       </c>
       <c r="D12" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>28</v>
       </c>
@@ -1500,10 +1501,10 @@
         <v>5</v>
       </c>
       <c r="D13" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>30</v>
       </c>
@@ -1514,24 +1515,24 @@
         <v>5</v>
       </c>
       <c r="D14" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
+        <v>135</v>
+      </c>
+      <c r="B15" t="s">
         <v>136</v>
-      </c>
-      <c r="B15" t="s">
-        <v>137</v>
       </c>
       <c r="C15" t="s">
         <v>5</v>
       </c>
       <c r="D15" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>32</v>
       </c>
@@ -1542,24 +1543,24 @@
         <v>5</v>
       </c>
       <c r="D16" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>34</v>
       </c>
       <c r="B17" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C17" t="s">
         <v>5</v>
       </c>
       <c r="D17" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>35</v>
       </c>
@@ -1573,7 +1574,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>35</v>
       </c>
@@ -1584,416 +1585,416 @@
         <v>12</v>
       </c>
       <c r="D19" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A20" t="s">
+      <c r="B20" t="s">
         <v>40</v>
-      </c>
-      <c r="B20" t="s">
-        <v>41</v>
       </c>
       <c r="C20" t="s">
         <v>5</v>
       </c>
       <c r="D20" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
+        <v>41</v>
+      </c>
+      <c r="B21" t="s">
         <v>42</v>
-      </c>
-      <c r="B21" t="s">
-        <v>43</v>
       </c>
       <c r="C21" t="s">
         <v>5</v>
       </c>
       <c r="D21" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
+        <v>43</v>
+      </c>
+      <c r="B22" t="s">
         <v>44</v>
-      </c>
-      <c r="B22" t="s">
-        <v>45</v>
       </c>
       <c r="C22" t="s">
         <v>5</v>
       </c>
       <c r="D22" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B23" t="s">
+        <v>45</v>
+      </c>
+      <c r="C23" t="s">
         <v>46</v>
       </c>
-      <c r="C23" t="s">
+      <c r="D23" t="s">
         <v>47</v>
       </c>
-      <c r="D23" t="s">
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A24" t="s">
+      <c r="B24" t="s">
         <v>49</v>
-      </c>
-      <c r="B24" t="s">
-        <v>50</v>
       </c>
       <c r="C24" t="s">
         <v>12</v>
       </c>
       <c r="D24" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B25" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C25" t="s">
         <v>12</v>
       </c>
       <c r="D25" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
+        <v>51</v>
+      </c>
+      <c r="B26" t="s">
         <v>52</v>
-      </c>
-      <c r="B26" t="s">
-        <v>53</v>
       </c>
       <c r="C26" t="s">
         <v>5</v>
       </c>
       <c r="D26" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
+        <v>102</v>
+      </c>
+      <c r="B27" t="s">
+        <v>53</v>
+      </c>
+      <c r="C27" t="s">
+        <v>54</v>
+      </c>
+      <c r="D27" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
         <v>103</v>
       </c>
-      <c r="B27" t="s">
-        <v>54</v>
-      </c>
-      <c r="C27" t="s">
-        <v>55</v>
-      </c>
-      <c r="D27" t="s">
+      <c r="B28" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A28" t="s">
-        <v>104</v>
-      </c>
-      <c r="B28" t="s">
+      <c r="C28" t="s">
+        <v>46</v>
+      </c>
+      <c r="D28" t="s">
         <v>57</v>
       </c>
-      <c r="C28" t="s">
-        <v>47</v>
-      </c>
-      <c r="D28" t="s">
+    </row>
+    <row r="29" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A29" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="B29" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A29" s="1" t="s">
-        <v>143</v>
-      </c>
-      <c r="B29" t="s">
+      <c r="D29" t="s">
         <v>59</v>
       </c>
-      <c r="D29" t="s">
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>141</v>
+      </c>
+      <c r="B30" t="s">
         <v>60</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A30" t="s">
-        <v>142</v>
-      </c>
-      <c r="B30" t="s">
-        <v>61</v>
       </c>
       <c r="C30" s="2">
         <v>4020</v>
       </c>
       <c r="D30" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>144</v>
+      </c>
+      <c r="B31" t="s">
         <v>62</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A31" t="s">
-        <v>145</v>
-      </c>
-      <c r="B31" t="s">
-        <v>63</v>
       </c>
       <c r="C31" s="2">
         <v>5020</v>
       </c>
       <c r="D31" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="E31" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
+        <v>132</v>
+      </c>
+      <c r="B32" t="s">
+        <v>63</v>
+      </c>
+      <c r="C32" t="s">
+        <v>64</v>
+      </c>
+      <c r="D32" t="s">
+        <v>153</v>
+      </c>
+      <c r="E32" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>66</v>
+      </c>
+      <c r="B33" t="s">
+        <v>67</v>
+      </c>
+      <c r="C33" t="s">
+        <v>68</v>
+      </c>
+      <c r="D33" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>70</v>
+      </c>
+      <c r="B34" t="s">
+        <v>71</v>
+      </c>
+      <c r="C34" t="s">
+        <v>68</v>
+      </c>
+      <c r="D34" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>73</v>
+      </c>
+      <c r="B35" t="s">
+        <v>74</v>
+      </c>
+      <c r="C35" t="s">
+        <v>64</v>
+      </c>
+      <c r="D35" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>104</v>
+      </c>
+      <c r="B36" t="s">
+        <v>76</v>
+      </c>
+      <c r="D36" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>105</v>
+      </c>
+      <c r="B37" t="s">
+        <v>78</v>
+      </c>
+      <c r="D37" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>106</v>
+      </c>
+      <c r="B38" t="s">
+        <v>80</v>
+      </c>
+      <c r="D38" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>157</v>
+      </c>
+      <c r="B39" t="s">
+        <v>82</v>
+      </c>
+      <c r="D39" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>107</v>
+      </c>
+      <c r="B40" t="s">
+        <v>83</v>
+      </c>
+      <c r="D40" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>130</v>
+      </c>
+      <c r="B41" t="s">
+        <v>85</v>
+      </c>
+      <c r="D41" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>150</v>
+      </c>
+      <c r="B42" t="s">
+        <v>87</v>
+      </c>
+      <c r="D42" t="s">
+        <v>149</v>
+      </c>
+      <c r="E42" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>108</v>
+      </c>
+      <c r="B43" t="s">
+        <v>88</v>
+      </c>
+      <c r="D43" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>134</v>
+      </c>
+      <c r="B44" t="s">
+        <v>90</v>
+      </c>
+      <c r="D44" t="s">
         <v>133</v>
       </c>
-      <c r="B32" t="s">
-        <v>64</v>
-      </c>
-      <c r="C32" t="s">
-        <v>65</v>
-      </c>
-      <c r="D32" t="s">
-        <v>154</v>
-      </c>
-      <c r="E32" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A33" t="s">
-        <v>67</v>
-      </c>
-      <c r="B33" t="s">
-        <v>68</v>
-      </c>
-      <c r="C33" t="s">
-        <v>69</v>
-      </c>
-      <c r="D33" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A34" t="s">
-        <v>71</v>
-      </c>
-      <c r="B34" t="s">
-        <v>72</v>
-      </c>
-      <c r="C34" t="s">
-        <v>69</v>
-      </c>
-      <c r="D34" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A35" t="s">
-        <v>74</v>
-      </c>
-      <c r="B35" t="s">
-        <v>75</v>
-      </c>
-      <c r="C35" t="s">
-        <v>65</v>
-      </c>
-      <c r="D35" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A36" t="s">
-        <v>105</v>
-      </c>
-      <c r="B36" t="s">
-        <v>77</v>
-      </c>
-      <c r="D36" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A37" t="s">
-        <v>106</v>
-      </c>
-      <c r="B37" t="s">
-        <v>79</v>
-      </c>
-      <c r="D37" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A38" t="s">
-        <v>107</v>
-      </c>
-      <c r="B38" t="s">
-        <v>81</v>
-      </c>
-      <c r="D38" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A39" t="s">
-        <v>158</v>
-      </c>
-      <c r="B39" t="s">
-        <v>83</v>
-      </c>
-      <c r="D39" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A40" t="s">
-        <v>108</v>
-      </c>
-      <c r="B40" t="s">
-        <v>84</v>
-      </c>
-      <c r="D40" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A41" t="s">
-        <v>131</v>
-      </c>
-      <c r="B41" t="s">
-        <v>86</v>
-      </c>
-      <c r="D41" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A42" t="s">
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>109</v>
+      </c>
+      <c r="B45" t="s">
+        <v>91</v>
+      </c>
+      <c r="D45" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>110</v>
+      </c>
+      <c r="B46" t="s">
+        <v>93</v>
+      </c>
+      <c r="D46" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>111</v>
+      </c>
+      <c r="B47" t="s">
+        <v>95</v>
+      </c>
+      <c r="D47" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>140</v>
+      </c>
+      <c r="B48" t="s">
+        <v>138</v>
+      </c>
+      <c r="D48" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>152</v>
+      </c>
+      <c r="B49" t="s">
+        <v>97</v>
+      </c>
+      <c r="D49" t="s">
         <v>151</v>
       </c>
-      <c r="B42" t="s">
-        <v>88</v>
-      </c>
-      <c r="D42" t="s">
-        <v>150</v>
-      </c>
-      <c r="E42" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A43" t="s">
-        <v>109</v>
-      </c>
-      <c r="B43" t="s">
-        <v>89</v>
-      </c>
-      <c r="D43" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A44" t="s">
-        <v>135</v>
-      </c>
-      <c r="B44" t="s">
-        <v>91</v>
-      </c>
-      <c r="D44" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A45" t="s">
-        <v>110</v>
-      </c>
-      <c r="B45" t="s">
-        <v>92</v>
-      </c>
-      <c r="D45" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A46" t="s">
-        <v>111</v>
-      </c>
-      <c r="B46" t="s">
-        <v>94</v>
-      </c>
-      <c r="D46" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A47" t="s">
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
         <v>112</v>
       </c>
-      <c r="B47" t="s">
-        <v>96</v>
-      </c>
-      <c r="D47" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A48" t="s">
-        <v>141</v>
-      </c>
-      <c r="B48" t="s">
-        <v>139</v>
-      </c>
-      <c r="D48" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A49" t="s">
-        <v>153</v>
-      </c>
-      <c r="B49" t="s">
+      <c r="B50" t="s">
         <v>98</v>
       </c>
-      <c r="D49" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A50" t="s">
+      <c r="D50" t="s">
+        <v>156</v>
+      </c>
+      <c r="E50" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
         <v>113</v>
       </c>
-      <c r="B50" t="s">
-        <v>99</v>
-      </c>
-      <c r="D50" t="s">
-        <v>157</v>
-      </c>
-      <c r="E50" t="s">
+      <c r="B51" t="s">
         <v>100</v>
       </c>
-    </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.55000000000000004">
-      <c r="A51" t="s">
-        <v>114</v>
-      </c>
-      <c r="B51" t="s">
-        <v>101</v>
-      </c>
       <c r="D51" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
   </sheetData>

</xml_diff>